<commit_message>
Apply horizontal field site cards
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for horizontal Research cards, Study topic cards, Notes card list, Field Sites cards, favicon/title changes, and skills table.</t>
+          <t>Recent jekyll build passed. Rendered output checked for Research grid cards, horizontal Field Sites cards, Study topic cards, Notes card list, favicon/title changes, and skills table.</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1085,7 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Horizontal card layout</t>
+          <t>Research card layout restored to compact grid</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>Changed from three-column cards to one horizontal card per row. Two tags shown per project.</t>
+          <t>Research cards were restored to the previous compact grid. Each card still links to a detail page and shows two tags.</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>Page rebuilt around actual sites and handled field data using categorized cards.</t>
+          <t>Page rebuilt around actual sites and handled field data using categorized horizontal cards.</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Added Study topic cards and Notes card list. Changed Research cards to horizontal one-per-row layout.</t>
+          <t>Added Study topic cards and Notes card list. Research temporarily changed to horizontal cards, later restored to grid.</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -2329,6 +2329,28 @@
       <c r="D9" s="11" t="inlineStr">
         <is>
           <t>Codex</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Field Sites horizontal cards correction</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Restored Research cards to the previous compact grid and applied the horizontal one-row card style to Field Sites instead.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Link field site cards and update ORCID
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for Research grid cards, horizontal Field Sites cards, Study topic cards, Notes card list, favicon/title changes, and skills table.</t>
+          <t>Recent jekyll build passed. Rendered output checked for Research grid cards, clickable horizontal Field Sites cards with detail pages, Study topic cards, Notes card list, favicon/title changes, ORCID link, and skills table.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>Page rebuilt around actual sites and handled field data using categorized horizontal cards.</t>
+          <t>Page rebuilt around actual sites and handled field data using categorized horizontal cards. Each card now links to a field-site detail page.</t>
         </is>
       </c>
     </row>
@@ -1298,6 +1298,38 @@
       <c r="F20" s="11" t="inlineStr">
         <is>
           <t>Done, Backlog, Next Actions, User Inputs, and Change Log updated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ORCID link correction</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Updated profile/sidebar ORCID URL to https://orcid.org/0000-0002-3527-8534.</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2354,6 +2386,28 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ORCID and clickable Field Sites update</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Updated ORCID link and converted Field Sites cards into links to per-site detail pages.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add PostgreSQL to skills
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -945,7 +945,7 @@
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Python, MATLAB, R, SQL, PyTorch, TensorFlow, scikit-learn, pandas/NumPy, Abaqus, LabVIEW, NI DIAdem, AWS, Docker, Git, Premiere Pro.</t>
+          <t>Python, MATLAB, R, C, JavaScript/Node.js, SQL, PostgreSQL, PyTorch, TensorFlow, scikit-learn, pandas/NumPy, Abaqus, Simulink, SolidWorks, Altium, LabVIEW, NI DIAdem, AWS, Docker, Git, Premiere Pro.</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2408,6 +2408,28 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Skills PostgreSQL update</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Added PostgreSQL to the tool-oriented skills table. LabVIEW was already included and remains listed under Measurement &amp; DAQ.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add field site image slots
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for Research grid cards, clickable horizontal Field Sites cards with detail pages, Study topic cards, Notes card list, favicon/title changes, ORCID link, and skills table.</t>
+          <t>Recent jekyll build passed. Rendered output checked for Research grid cards, clickable horizontal Field Sites cards with left image slots and detail pages, Study topic cards, Notes card list, favicon/title changes, ORCID link, and skills table.</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>SHM, WIM/OBM, IoT sensing, AI-based data analysis, and field bridge monitoring experience reflected.</t>
+          <t>SHM, WIM/OBM, IoT sensing, AI-based data analysis, AI for Physical Systems, and field bridge monitoring experience reflected.</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>Page rebuilt around actual sites and handled field data using categorized horizontal cards. Each card now links to a field-site detail page.</t>
+          <t>Page rebuilt around actual sites and handled field data using categorized horizontal cards. Each card links to a field-site detail page and now includes a left image slot for future site photos.</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>Useful for WIM, OBM, Bridge Monitoring, Portable Sensing, and Field Sites pages.</t>
+          <t>Useful for WIM, OBM, Bridge Monitoring, Portable Sensing, and Field Sites cards/detail pages.</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2430,6 +2430,28 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Field Sites image slots and AI keyword update</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Added left-side image slots to clickable Field Sites cards and replaced AI-based Signal Interpretation with AI for Physical Systems.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refine field sites and project metadata
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for Research grid cards, clickable horizontal Field Sites cards with left image slots and detail pages, Study topic cards, Notes card list, favicon/title changes, ORCID link, and skills table.</t>
+          <t>Recent jekyll build passed. Rendered output checked for Research grid cards, clickable Field Sites cards with left image slots and detail pages, Study topic cards, Notes card list, favicon/title changes, ORCID link, and skills table.</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>SHM, WIM/OBM, IoT sensing, AI-based data analysis, AI for Physical Systems, and field bridge monitoring experience reflected.</t>
+          <t>SHM, WIM/OBM, IoT sensing, AI-based data analysis, AI for Physical Systems, field bridge monitoring experience, and simplified sidebar degree reflected.</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>Research cards were restored to the previous compact grid. Each card still links to a detail page and shows two tags.</t>
+          <t>Research cards use the compact grid. Smart Concrete Sensing System period corrected to 2020-2021. Each card links to a detail page and shows two tags.</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>Page rebuilt around actual sites and handled field data using categorized horizontal cards. Each card links to a field-site detail page and now includes a left image slot for future site photos.</t>
+          <t>Page rebuilt around actual sites and handled field data using clickable cards with left image slots and per-site detail pages. Intro text shortened.</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>After deployment, check favicon/title, Research horizontal cards, Study/Notes cards, and Field Sites cards in Chrome and mobile width.</t>
+          <t>After deployment, check favicon/title, Research grid cards, Field Sites image cards, Study/Notes cards, and mobile width behavior in Chrome.</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
@@ -2157,7 +2157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2452,6 +2452,28 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Field Sites intro and Smart Concrete period update</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Shortened Field Sites intro, corrected Smart Concrete Sensing System period to 2020-2021, and simplified sidebar degree text.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add thesis button and funding section
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1333,6 +1333,70 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Funded Research placeholder section</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Added a Funded Research section at the bottom of Research, backed by _data/funding.yml for future entries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Read Thesis button placeholder</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Added a disabled Read Thesis pill beside the M.S. degree line. It can be turned into a PDF link once the thesis file is available.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1345,7 +1409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1705,6 +1769,38 @@
       <c r="F11" s="11" t="inlineStr">
         <is>
           <t>Check indexing status of important URLs and sitemap submission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Upload M.S. thesis PDF</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>User needed</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Add the actual thesis PDF to assets/files, then convert the Read Thesis placeholder into a working link.</t>
         </is>
       </c>
     </row>
@@ -1919,7 +2015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -2142,6 +2238,33 @@
       <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Chrome may cache favicon. Screenshots help if spacing or icon updates look stale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>M.S. thesis PDF</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Required for active thesis link</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>User needed</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Needed to make the Read Thesis button open an actual PDF instead of remaining disabled.</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2474,6 +2597,28 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Thesis button and funding placeholder</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Added a disabled Read Thesis pill beside the M.S. degree and created a Funded Research section backed by funding.yml.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Link master thesis PDF
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -1373,7 +1373,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Read Thesis button placeholder</t>
+          <t>Read Thesis PDF link</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Added a disabled Read Thesis pill beside the M.S. degree line. It can be turned into a PDF link once the thesis file is available.</t>
+          <t>Added Junyoung_Park_Master_Thesis.pdf and connected the Read Thesis pill beside the M.S. degree line.</t>
         </is>
       </c>
     </row>
@@ -1785,7 +1785,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>User needed</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1800,7 +1800,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Add the actual thesis PDF to assets/files, then convert the Read Thesis placeholder into a working link.</t>
+          <t>Completed. PDF is available at assets/files/Junyoung_Park_Master_Thesis.pdf.</t>
         </is>
       </c>
     </row>
@@ -2254,7 +2254,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>User needed</t>
+          <t>Received</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Needed to make the Read Thesis button open an actual PDF instead of remaining disabled.</t>
+          <t>Received and linked as assets/files/Junyoung_Park_Master_Thesis.pdf.</t>
         </is>
       </c>
     </row>
@@ -2280,7 +2280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2619,6 +2619,28 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>M.S. thesis PDF linked</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Copied the master thesis PDF into assets/files and connected the Read Thesis button on About and CV.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Move funding to project pages
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -1105,7 +1105,7 @@
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>Research cards use the compact grid. Smart Concrete Sensing System period corrected to 2020-2021. Each card links to a detail page and shows two tags.</t>
+          <t>Research cards use the compact grid. Added Sewer Monitoring Sensor System under Smart Sensing Systems and kept project cards linked to detail pages.</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Funded Research placeholder section</t>
+          <t>Project-level Funded by placeholders</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Added a Funded Research section at the bottom of Research, backed by _data/funding.yml for future entries.</t>
+          <t>Removed the global Research funding section and added Funded by placeholders to each project detail page using _data/project_funding.yml.</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1393,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Added Junyoung_Park_Master_Thesis.pdf and connected the Read Thesis pill beside the M.S. degree line.</t>
+          <t>Read Thesis now appears beside the M.S. dissertation title and opens Junyoung_Park_Master_Thesis.pdf.</t>
         </is>
       </c>
     </row>
@@ -1460,12 +1460,12 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Decide whether to add participated/funded research projects</t>
+          <t>Fill project-level Funded by entries</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>User needed</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="F2" s="11" t="inlineStr">
         <is>
-          <t>Recommended if official project title, English title, period, funding/host agency, role, and contribution can be listed.</t>
+          <t>Add funder names, periods, and roles for each project in _data/project_funding.yml when the funding list is ready.</t>
         </is>
       </c>
     </row>
@@ -1884,12 +1884,12 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>Design a Research Projects section</t>
+          <t>Fill project-level funding data</t>
         </is>
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
-          <t>After info is collected, decide whether it belongs near the top or bottom of Research and whether to use cards or timeline rows.</t>
+          <t>Use _data/project_funding.yml to add funders per project detail page; no separate Research-wide funding section is currently needed.</t>
         </is>
       </c>
       <c r="D3" s="11" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>After data is available</t>
+          <t>After funding list is ready</t>
         </is>
       </c>
     </row>
@@ -2055,12 +2055,12 @@
     <row r="2" ht="54" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Participated research project list</t>
+          <t>Project-level funding details</t>
         </is>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Required for next Research update</t>
+          <t>Required for Funded by sections</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>Title KR/EN, period, funding or host agency, role, contribution, and public/confidential status.</t>
+          <t>For each project: funder/agency name, period, role, and whether it can be publicly shown.</t>
         </is>
       </c>
     </row>
@@ -2280,7 +2280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2641,6 +2641,28 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Project-level funding and sewer sensor update</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Moved funding placeholders from Research index to each project detail page, added Sewer Monitoring Sensor System, and moved Read Thesis beside the dissertation title.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update favicon and hobbies
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>694f981 Refine research and notes layout. This checklist update is the next tracked change.</t>
+          <t>9702571 Move funding to project pages. This checklist update adds the 📡 favicon and PKM hobby refinement.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for Research grid cards, clickable Field Sites cards with left image slots and detail pages, Study topic cards, Notes card list, favicon/title changes, ORCID link, and skills table.</t>
+          <t>Recent jekyll build passed. Rendered output checked for Research grid cards, clickable Field Sites cards with left image slots and detail pages, Study topic cards, Notes card list, 📡 favicon cache-busted link, ORCID link, skills table, and About hobby chips.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1394,6 +1394,70 @@
       <c r="F23" t="inlineStr">
         <is>
           <t>Read Thesis now appears beside the M.S. dissertation title and opens Junyoung_Park_Master_Thesis.pdf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Site chrome</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>📡 favicon update</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Replaced the SVG favicon with a radar emoji and added cache-busting query strings to favicon links.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>About</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>PKM hobby chip</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Added 🧠 PKM to the Hobbies chip list next to Swimming and Drumming.</t>
         </is>
       </c>
     </row>
@@ -2280,7 +2344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2663,6 +2727,28 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Favicon and hobbies update</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Changed the browser/site favicon to 📡, added favicon cache busting, and added 🧠 PKM under Hobbies.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refine theme profile and research interests
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>9702571 Move funding to project pages. This checklist update adds the 📡 favicon and PKM hobby refinement.</t>
+          <t>d1854bb Update favicon and hobbies. This checklist update covers light-mode default, profile location, and Research Interests wording.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for Research grid cards, clickable Field Sites cards with left image slots and detail pages, Study topic cards, Notes card list, 📡 favicon cache-busted link, ORCID link, skills table, and About hobby chips.</t>
+          <t>Recent jekyll build passed. Rendered output checked for default light theme script, sidebar Seoul location, Research Interests wording, Research grid cards, Field Sites cards, favicon, ORCID link, and skills table.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1458,6 +1458,102 @@
       <c r="F25" t="inlineStr">
         <is>
           <t>Added 🧠 PKM to the Hobbies chip list next to Swimming and Drumming.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Default light mode</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Changed first-visit/incognito behavior to use light mode unless the visitor has explicitly saved dark mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Seoul location marker</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Added Seoul, South Korea to the sidebar profile card with a location marker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>About/CV</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Research Interests wording cleanup</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Reorganized the three explanatory bullets into Infrastructure Monitoring, Sensing &amp; Measurement Systems, and AI for Engineering Data.</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2749,6 +2845,28 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Theme and research interests refinement</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Set the site default to light mode, added Seoul to the profile card, and unified the Research Interests explanatory bullets on About and CV.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Align layout and simplify research cards
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>f572ff2 Refine theme profile and research interests. This checklist update covers profile card framing and sharper Research Interests positioning.</t>
+          <t>d97c1b6 Strengthen research positioning. This checklist update covers global layout rhythm, simplified Research cards, and a cleaner About page structure.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for default light theme, sidebar Seoul location, framed profile card, updated Research Interests wording, Research grid cards, Field Sites cards, favicon, ORCID link, and skills table.</t>
+          <t>Recent jekyll build passed. Rendered output checked for aligned site/profile start, sticky profile behavior, simplified Research cards without period/tag chips, markdown-style About sections, favicon, ORCID link, and skills table.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1618,6 +1618,102 @@
       <c r="F30" t="inlineStr">
         <is>
           <t>Reframed the three bullets as Field-Validated Infrastructure Intelligence, Deployable Sensing &amp; Edge-to-Cloud Measurement, and Physics-Aware AI for Engineering Systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Layout</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Unified page start rhythm</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Adjusted topbar height, site top padding, grid alignment, and sticky profile offset so page titles and the profile card start consistently.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Simplified project cards</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Removed period and tag chips from Research cards; cards now show title, image area, and concise summary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>About</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Cleaner markdown-style structure</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Converted About education and work experience sections from custom entry blocks to a simpler markdown-like presentation.</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2953,6 +3049,28 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Layout rhythm and Research cards</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Aligned page/profile vertical rhythm, kept the profile sticky, simplified Research cards, and cleaned the About page section structure.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Restore research cards and update favicon assets
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>d97c1b6 Strengthen research positioning. This checklist update covers global layout rhythm, simplified Research cards, and a cleaner About page structure.</t>
+          <t>4d5d3fb Align layout and simplify research cards. This checklist update corrects Research card metadata and updates PNG/ICO favicon assets for the Chrome tab.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for aligned site/profile start, sticky profile behavior, simplified Research cards without period/tag chips, markdown-style About sections, favicon, ORCID link, and skills table.</t>
+          <t>Recent jekyll build passed. Rendered output checked for aligned site/profile start, sticky profile behavior, Research cards with period and two tag chips, markdown-style About sections, SVG/PNG/ICO favicon assets, ORCID link, and skills table.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Removed period and tag chips from Research cards; cards now show title, image area, and concise summary.</t>
+          <t>Restored period and two representative tag chips on Research cards after correction; cards show image area, title, period, summary, and tags.</t>
         </is>
       </c>
     </row>
@@ -1714,6 +1714,70 @@
       <c r="F33" t="inlineStr">
         <is>
           <t>Converted About education and work experience sections from custom entry blocks to a simpler markdown-like presentation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Restore project card period and tags</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Restored year/period and two representative tag chips on Research project cards after the previous overreach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Site chrome</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Chrome tab favicon assets</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Regenerated favicon PNG and ICO assets so Chrome can show the radar icon even when it uses non-SVG favicon files.</t>
         </is>
       </c>
     </row>
@@ -2600,7 +2664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3062,10 +3126,54 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Aligned page/profile vertical rhythm, kept the profile sticky, simplified Research cards, and cleaned the About page section structure.</t>
+          <t>Aligned page/profile vertical rhythm, kept the profile sticky, kept Research card period/tag chips after correction, and cleaned the About page section structure.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Research card correction</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Restored the Research project card period and two tag chips; this corrects the previous unintended removal.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Chrome tab favicon assets</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Regenerated favicon-32x32, favicon-192x192, favicon-512x512, favicon.ico, and apple-touch-icon with the radar icon.</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
         <is>
           <t>User + Codex</t>
         </is>

</xml_diff>

<commit_message>
Update favicon to galaxy icon
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>4d5d3fb Align layout and simplify research cards. This checklist update corrects Research card metadata and updates PNG/ICO favicon assets for the Chrome tab.</t>
+          <t>bbcbfc3 Restore research cards and update favicon assets. This checklist update changes all favicon assets to the galaxy icon and adds a root favicon.ico for loading state.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for aligned site/profile start, sticky profile behavior, Research cards with period and two tag chips, markdown-style About sections, SVG/PNG/ICO favicon assets, ORCID link, and skills table.</t>
+          <t>Recent jekyll build passed. Rendered output checked for root favicon.ico, SVG/PNG/ICO galaxy favicon assets, cache-busted favicon links, Research cards with period and two tag chips, aligned layout rhythm, ORCID link, and skills table.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1778,6 +1778,38 @@
       <c r="F35" t="inlineStr">
         <is>
           <t>Regenerated favicon PNG and ICO assets so Chrome can show the radar icon even when it uses non-SVG favicon files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Site chrome</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Galaxy favicon loading state</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Changed SVG, PNG, ICO, apple-touch, and root favicon.ico assets to the galaxy icon so Chrome can use it during loading and after load.</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3179,6 +3211,28 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Galaxy favicon update</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Changed the Chrome tab favicon from radar to galaxy across SVG, PNG, ICO, apple-touch, and root favicon.ico assets, with cache-busted links.</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add concrete field site locations
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>42790bd Restore research interests heading. This checklist update removes the extra light favicon backing and keeps the galaxy icon transparent.</t>
+          <t>b5924e3 Remove favicon backing. This checklist update adds the latest Field Sites list from user-provided site names.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for transparent galaxy favicon SVG, root favicon.ico, matching image favicon.ico, cache-busted favicon links, ORCID link, and skills table.</t>
+          <t>Recent jekyll build passed. Rendered output checked for Field Sites cards/detail pages, Cheongdam 1 Bridge page, Saemangeum/Bongdong WIM sites, freight bearing monitoring, Cheonma Remicon, Incheon Port, transparent galaxy favicon, ORCID link, and skills table.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1845,6 +1845,70 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Add user-provided site names</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Updated Field Sites with Seongsan, Seosomun, Paldang, Cheongdam 1 Bridge, Saemangeum/Bongdong WIM, Koryeo Hwacha freight bearing monitoring, Cheonma Remicon, and Incheon Port.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Sites section on cards/details</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Added a Sites list to Field Sites cards and detail pages so concrete field locations are visible before data types.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1857,7 +1921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2249,6 +2313,38 @@
       <c r="F12" t="inlineStr">
         <is>
           <t>Completed. PDF is available at assets/files/Junyoung_Park_Master_Thesis.pdf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Add field-site photos</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>User needed</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Add public/non-confidential images for Seongsan, Seosomun, Paldang, Cheongdam 1 Bridge, Saemangeum, Bongdong, Koryeo Hwacha, Cheonma Remicon, and Incheon Port.</t>
         </is>
       </c>
     </row>
@@ -2728,7 +2824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3287,6 +3383,28 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Field Sites concrete site update</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Added the user-provided field site names to Field Sites cards/detail pages and replaced the generic bridge campaigns page with Cheongdam 1 Bridge.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refine field site locations
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>b5924e3 Remove favicon backing. This checklist update adds the latest Field Sites list from user-provided site names.</t>
+          <t>dabbaa6 Add concrete field site locations. This checklist update corrects the prefabricated field site to Seoul bus-only lane, adds known location labels, and refines the About page Education/Work Experience layout.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for Field Sites cards/detail pages, Cheongdam 1 Bridge page, Saemangeum/Bongdong WIM sites, freight bearing monitoring, Cheonma Remicon, Incheon Port, transparent galaxy favicon, ORCID link, and skills table.</t>
+          <t>Recent jekyll build passed. Rendered output checked for Field Sites cards/detail pages, location labels, Seoul bus-only lane prefabricated monitoring, removal of Cheonma Remicon, About page summary entries, transparent galaxy favicon, ORCID link, and skills table.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Updated Field Sites with Seongsan, Seosomun, Paldang, Cheongdam 1 Bridge, Saemangeum/Bongdong WIM, Koryeo Hwacha freight bearing monitoring, Cheonma Remicon, and Incheon Port.</t>
+          <t>Updated Field Sites with Seongsan, Seosomun, Paldang, Cheongdam 1 Bridge, Saemangeum/Bongdong WIM, Koryeo Hwacha freight bearing monitoring, Seoul bus-only lane transportation monitoring, and Incheon Port.</t>
         </is>
       </c>
     </row>
@@ -1906,6 +1906,102 @@
       <c r="F39" t="inlineStr">
         <is>
           <t>Added a Sites list to Field Sites cards and detail pages so concrete field locations are visible before data types.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Add location labels</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Added known location labels for bridge, WIM, Seoul bus-only lane, and Incheon Port field sites; left uncertain locations broad or blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Correct prefabricated field site</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Replaced Cheonma Remicon with Seoul Bus-Only Lane Transportation Monitoring in Field Sites cards and the detail page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>About</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Refine Education and Work Experience layout</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Changed the About page Education and Work Experience sections from plain markdown blocks to compact dated summary entries.</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3405,6 +3501,28 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Field Sites locations and About layout</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Added known field-site locations, corrected the prefabricated field site to Seoul bus-only lane monitoring, removed Cheonma Remicon from rendered content, and refined About page Education/Work Experience entries.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Polish bilingual research layout
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>dabbaa6 Add concrete field site locations. This checklist update corrects the prefabricated field site to Seoul bus-only lane, adds known location labels, and refines the About page Education/Work Experience layout.</t>
+          <t>783c5ee Refine field site locations. This checklist update adds bilingual Research project taxonomy, refines the About page, adjusts Publications metadata/buttons, and adds a sticky-bottom footer.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for Field Sites cards/detail pages, location labels, Seoul bus-only lane prefabricated monitoring, removal of Cheonma Remicon, About page summary entries, transparent galaxy favicon, ORCID link, and skills table.</t>
+          <t>Recent jekyll build passed. Rendered output checked for bilingual Research headings/cards, Soongsil project page, About bilingual intro/coursework/contact, Publications tag/action placement, and footer placement on Study/Notes.</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>1) Organize participated research projects 2) Add public images/results to representative project detail pages 3) Write the next Study or Notes post 4) Replace the CV PDF with the latest file.</t>
+          <t>1) Fill representative Research project pages with concrete figures, field photos, and outcomes 2) Add exact funding entries per project 3) Add 1-2 Study/Notes posts 4) Replace the CV PDF with the latest file.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2002,6 +2002,134 @@
       <c r="F42" t="inlineStr">
         <is>
           <t>Changed the About page Education and Work Experience sections from plain markdown blocks to compact dated summary entries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Add bilingual project taxonomy</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Added Korean and English group/project labels to Research cards and added the Soongsil University Structural Monitoring System entry/page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>About</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Restore bilingual intro and CV-like sections</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Restored English/Korean intro text, changed About Education/Work Experience back to CV-style entries, kept coursework, and added Contact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Publications</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Move project actions below tags</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Limited visible publication tags to two, kept Source Document hidden because titles are links, and moved Project actions below tags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Layout</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Add bottom footer</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Added a footer with contact/profile links and flex layout so short Study/Notes pages keep the footer at the bottom.</t>
         </is>
       </c>
     </row>
@@ -2920,7 +3048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3523,6 +3651,28 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Bilingual Research and About/Publications polish</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Added bilingual Research cards, restored bilingual About intro with Contact, refined Publications tags/actions, and added a site footer for short pages.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Revert "Polish bilingual research layout"
This reverts commit 93b6275126b0701e3ce282dc79bfdfdf188cb029.
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>783c5ee Refine field site locations. This checklist update adds bilingual Research project taxonomy, refines the About page, adjusts Publications metadata/buttons, and adds a sticky-bottom footer.</t>
+          <t>dabbaa6 Add concrete field site locations. This checklist update corrects the prefabricated field site to Seoul bus-only lane, adds known location labels, and refines the About page Education/Work Experience layout.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for bilingual Research headings/cards, Soongsil project page, About bilingual intro/coursework/contact, Publications tag/action placement, and footer placement on Study/Notes.</t>
+          <t>Recent jekyll build passed. Rendered output checked for Field Sites cards/detail pages, location labels, Seoul bus-only lane prefabricated monitoring, removal of Cheonma Remicon, About page summary entries, transparent galaxy favicon, ORCID link, and skills table.</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>1) Fill representative Research project pages with concrete figures, field photos, and outcomes 2) Add exact funding entries per project 3) Add 1-2 Study/Notes posts 4) Replace the CV PDF with the latest file.</t>
+          <t>1) Organize participated research projects 2) Add public images/results to representative project detail pages 3) Write the next Study or Notes post 4) Replace the CV PDF with the latest file.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2002,134 +2002,6 @@
       <c r="F42" t="inlineStr">
         <is>
           <t>Changed the About page Education and Work Experience sections from plain markdown blocks to compact dated summary entries.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Add bilingual project taxonomy</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>User + Codex</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Added Korean and English group/project labels to Research cards and added the Soongsil University Structural Monitoring System entry/page.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>About</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Restore bilingual intro and CV-like sections</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>User + Codex</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Restored English/Korean intro text, changed About Education/Work Experience back to CV-style entries, kept coursework, and added Contact.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Publications</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Move project actions below tags</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>User + Codex</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Limited visible publication tags to two, kept Source Document hidden because titles are links, and moved Project actions below tags.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Layout</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Add bottom footer</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>User + Codex</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Added a footer with contact/profile links and flex layout so short Study/Notes pages keep the footer at the bottom.</t>
         </is>
       </c>
     </row>
@@ -3048,7 +2920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3651,28 +3523,6 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2026-05-16</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Bilingual Research and About/Publications polish</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Added bilingual Research cards, restored bilingual About intro with Contact, refined Publications tags/actions, and added a site footer for short pages.</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>User + Codex</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sharpen PhD contact positioning
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>dabbaa6 Add concrete field site locations. This checklist update corrects the prefabricated field site to Seoul bus-only lane, adds known location labels, and refines the About page Education/Work Experience layout.</t>
+          <t>cd25046 Revert "Polish bilingual research layout". This checklist update sharpens the About-page contact message and Research Fit language for prospective PhD advisors.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for Field Sites cards/detail pages, location labels, Seoul bus-only lane prefabricated monitoring, removal of Cheonma Remicon, About page summary entries, transparent galaxy favicon, ORCID link, and skills table.</t>
+          <t>Recent jekyll build passed. Rendered output checked for the new About lead sentence, Research Fit bullets, and Research page intro copy.</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>1) Organize participated research projects 2) Add public images/results to representative project detail pages 3) Write the next Study or Notes post 4) Replace the CV PDF with the latest file.</t>
+          <t>1) Update the CV PDF when the user provides the new version 2) Add field photos/plots/results to representative Research detail pages 3) Add concise role/outcome blocks to Field Sites 4) Keep professor-specific contact links in email drafts rather than overloading the homepage.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2002,6 +2002,70 @@
       <c r="F42" t="inlineStr">
         <is>
           <t>Changed the About page Education and Work Experience sections from plain markdown blocks to compact dated summary entries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>About</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Sharpen PhD contact positioning</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Added a memorable lead sentence and Research Fit bullets for AI/digital twin/reliability, smart sensing/IoT, and vehicle-bridge/transportation monitoring groups.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Align Research page intro with contact positioning</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Updated the Research page intro to emphasize deployable sensing systems, field data, and engineering interpretation.</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3523,6 +3587,28 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PhD contact positioning copy</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Sharpened the About lead sentence, added Research Fit bullets for prospective advisor audiences, and aligned the Research page intro.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Improve mobile navigation layout
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>60c03ee Sharpen PhD contact positioning. This checklist update replaces the downloadable CV PDF with the May 2026 version.</t>
+          <t>4243bea Update downloadable CV. This checklist update improves the mobile navigation and profile-card layout while preserving the desktop layout.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for CV download link, Last updated: May 2026 label, and the updated PDF copied into the build output.</t>
+          <t>Recent jekyll build passed. Rendered output checked for the mobile nav toggle markup/script, collapsed mobile menu CSS, and compact mobile profile-card styling.</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>1) Review whether the web CV page content should be synchronized line-by-line with the new PDF 2) Add field photos/plots/results to representative Research detail pages 3) Add concise role/outcome blocks to Field Sites 4) Prepare professor-specific contact email drafts.</t>
+          <t>1) Review the live mobile page after GitHub Pages deploy 2) Add field photos/plots/results to representative Research detail pages 3) Add concise role/outcome blocks to Field Sites 4) Prepare professor-specific contact email drafts.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2098,6 +2098,70 @@
       <c r="F45" t="inlineStr">
         <is>
           <t>Replaced assets/files/Junyoung_Park_CV.pdf with CV_Junyoung_Park_2026_v1.pdf and updated the CV page label to May 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Mobile UI</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Add collapsible mobile navigation</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Added a mobile-only menu toggle that collapses the navigation on narrow screens while preserving the desktop navbar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Mobile UI</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Compact mobile profile card</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Changed the mobile profile card to a smaller horizontal layout with reduced photo size and compact links.</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3663,6 +3727,28 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Mobile navigation and profile layout</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Added a mobile menu toggle and compact mobile profile-card styling without changing the desktop layout.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Standardize research project pages
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>4243bea Update downloadable CV. This checklist update improves the mobile navigation and profile-card layout while preserving the desktop layout.</t>
+          <t>361e196 Improve mobile navigation layout. This checklist update standardizes Research project detail pages and updates advisor wording.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for the mobile nav toggle markup/script, collapsed mobile menu CSS, and compact mobile profile-card styling.</t>
+          <t>Recent jekyll build passed. Rendered output checked for standardized project-detail headings and the late Jongwoong Park advisor wording on About/CV.</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>1) Review the live mobile page after GitHub Pages deploy 2) Add field photos/plots/results to representative Research detail pages 3) Add concise role/outcome blocks to Field Sites 4) Prepare professor-specific contact email drafts.</t>
+          <t>1) Add project-specific images/plots to the standardized Research detail pages 2) Add concise role/outcome blocks to Field Sites 3) Review whether Related Publications / Outputs should link directly to Publications entries 4) Prepare professor-specific contact email drafts.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2162,6 +2162,70 @@
       <c r="F47" t="inlineStr">
         <is>
           <t>Changed the mobile profile card to a smaller horizontal layout with reduced photo size and compact links.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Standardize project detail pages</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Updated all Research project detail pages to use Problem, My Role, System / Methods, Field Deployment, Data / Outputs, and Related Publications / Outputs sections.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>About/CV</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Update advisor wording</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Changed the advisor line to the late Jongwoong Park on About and CV pages.</t>
         </is>
       </c>
     </row>
@@ -3080,7 +3144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3749,6 +3813,28 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Standardized Research detail pages</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Reworked all Research project detail pages into a consistent structure and updated advisor wording to the late Jongwoong Park.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update CV skills and talks
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>361e196 Improve mobile navigation layout. This checklist update standardizes Research project detail pages and updates advisor wording.</t>
+          <t>05cd652 Standardize research project pages. This checklist update replaces the downloadable CV with v2, syncs Skills with the CV, and splits Talks into international/domestic conference sections.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for standardized project-detail headings and the late Jongwoong Park advisor wording on About/CV.</t>
+          <t>Recent jekyll build passed. Rendered output checked for CV v2 PDF size/date, CV-aligned Skills table, and International/Domestic Conference sections on Talks.</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>1) Add project-specific images/plots to the standardized Research detail pages 2) Add concise role/outcome blocks to Field Sites 3) Review whether Related Publications / Outputs should link directly to Publications entries 4) Prepare professor-specific contact email drafts.</t>
+          <t>1) Add project-specific images/plots to standardized Research detail pages 2) Add concise role/outcome blocks to Field Sites 3) Review whether Related Publications / Outputs should link directly to Publications entries 4) Prepare professor-specific contact email drafts.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2226,6 +2226,102 @@
       <c r="F49" t="inlineStr">
         <is>
           <t>Changed the advisor line to the late Jongwoong Park on About and CV pages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>CV</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Replace downloadable CV with v2</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Replaced assets/files/Junyoung_Park_CV.pdf with CV_Junyoung_Park_2026_v2.pdf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Skills</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Sync skills table with CV</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Updated the homepage/CV skills table to match the Programming, ML, Software, Data, and Languages groups in the new CV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Talks</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Split conference presentations</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Separated Talks into International Conferences and Domestic Conferences using the existing venue classification.</t>
         </is>
       </c>
     </row>
@@ -3144,7 +3240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3835,6 +3931,28 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>CV v2, skills, and Talks split</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Replaced the downloadable CV with v2, synced the Skills table with the CV, and split Talks into international/domestic conference sections.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add project figure editing guide
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll build passed. Rendered output checked for CV v2 PDF size/date, CV-aligned Skills table, and International/Domestic Conference sections on Talks.</t>
+          <t>Recent jekyll clean + jekyll build passed. Checked that CONTENT_EDITING_GUIDE.md is excluded from _site and project figure CSS is present in the built CSS.</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>1) Add project-specific images/plots to standardized Research detail pages 2) Add concise role/outcome blocks to Field Sites 3) Review whether Related Publications / Outputs should link directly to Publications entries 4) Prepare professor-specific contact email drafts.</t>
+          <t>1) Add actual project images/plots to images/projects/&lt;project-key&gt;/ 2) Insert figure blocks in the relevant project Markdown pages 3) Link Related Publications / Outputs to Publications entries 4) Prepare professor-specific contact email drafts.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2322,6 +2322,102 @@
       <c r="F52" t="inlineStr">
         <is>
           <t>Separated Talks into International Conferences and Domestic Conferences using the existing venue classification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Add project figure styling</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Added reusable project figure and figure-grid CSS so project pages can display field photos, diagrams, and plots cleanly when content is added.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Assets</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Create project image folders</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Added images/projects/&lt;project-key&gt;/ folders with .gitkeep placeholders for research project images and plots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Add content editing guide</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Added CONTENT_EDITING_GUIDE.md explaining where to edit project text, where to store images, and how to reference figures in Markdown/HTML.</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3336,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3953,6 +4049,28 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Project image folders and editing guide</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Added project image folders, reusable project figure CSS, and a local content editing guide for future writing/image work.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Document notes and study writing workflow
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -598,7 +598,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Recent jekyll clean + jekyll build passed. Checked that CONTENT_EDITING_GUIDE.md is excluded from _site and project figure CSS is present in the built CSS.</t>
+          <t>Recent jekyll build passed. Checked that CONTENT_EDITING_GUIDE.md is excluded from _site and content/project figure CSS is present in the built CSS.</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>1) Add actual project images/plots to images/projects/&lt;project-key&gt;/ 2) Insert figure blocks in the relevant project Markdown pages 3) Link Related Publications / Outputs to Publications entries 4) Prepare professor-specific contact email drafts.</t>
+          <t>1) Add actual project images/plots to images/projects/&lt;project-key&gt;/ 2) Draft Notes or Study posts in _posts/ using CONTENT_EDITING_GUIDE.md 3) Link Related Publications / Outputs to Publications entries 4) Prepare professor-specific contact email drafts.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2418,6 +2418,70 @@
       <c r="F55" t="inlineStr">
         <is>
           <t>Added CONTENT_EDITING_GUIDE.md explaining where to edit project text, where to store images, and how to reference figures in Markdown/HTML.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Extend writing guide for Notes and Study</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Expanded CONTENT_EDITING_GUIDE.md with Notes/Study post file paths, front matter examples, image paths, and figure snippets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Assets</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Create Notes and Study image folders</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Added images/notes/ and images/study/ folders for post-specific figures and study images.</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4071,6 +4135,28 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Notes and Study writing guide</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Added instructions for writing Notes and Study posts, including front matter, image folders, and reusable figure markup.</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Embed Seongsan monitoring dashboard video
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2514,6 +2514,38 @@
       <c r="F58" t="inlineStr">
         <is>
           <t>Reduced the Study page to a modest intro, three current topics, and the existing study notes list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Embed Seongsan dashboard demonstration video</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Added a YouTube dashboard demonstration embed to the Cloud-Based Long-Term Bridge Monitoring System project page.</t>
         </is>
       </c>
     </row>
@@ -3432,7 +3464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4211,6 +4243,28 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Embedded Seongsan monitoring dashboard video</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Added the real-time Seongsan Bridge monitoring dashboard YouTube video to the bridge monitoring project page with responsive video styling.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refine field sites layout
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2546,6 +2546,70 @@
       <c r="F59" t="inlineStr">
         <is>
           <t>Added a YouTube dashboard demonstration embed to the Cloud-Based Long-Term Bridge Monitoring System project page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Refine field site information structure</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Reworked Field Sites cards and detail pages to use field focus, measurements/outputs, and compact metadata instead of repetitive Location/Sites/Data handled sections.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Embed Seongsan dashboard video on field site page</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Added the Seongsan Bridge real-time monitoring dashboard YouTube embed to the Seongsan Bridge field site detail page.</t>
         </is>
       </c>
     </row>
@@ -3464,7 +3528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4265,6 +4329,28 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Refined Field Sites layout and Seongsan video</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Updated Field Sites card/detail terminology, moved location into compact metadata, removed redundant single-site listings, and embedded the Seongsan dashboard video.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Simplify field site cards
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2610,6 +2610,38 @@
       <c r="F61" t="inlineStr">
         <is>
           <t>Added the Seongsan Bridge real-time monitoring dashboard YouTube embed to the Seongsan Bridge field site detail page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Simplify field site card layout</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Changed Field Sites listing cards to a larger landscape image plus concise right-side title/summary, removing the crowded details column from the list view.</t>
         </is>
       </c>
     </row>
@@ -3528,7 +3560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4351,6 +4383,28 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Simplified Field Sites cards</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Made field site list cards more image-led and removed the extra details column from the card view.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add field site card summaries
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2642,6 +2642,38 @@
       <c r="F62" t="inlineStr">
         <is>
           <t>Changed Field Sites listing cards to a larger landscape image plus concise right-side title/summary, removing the crowded details column from the list view.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Add period and data summaries to field site cards</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Updated Field Sites cards with a divider, blue site title, orange field-period label, period line, and concise data-summary text.</t>
         </is>
       </c>
     </row>
@@ -3560,7 +3592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4405,6 +4437,28 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Added field period and data summaries to cards</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Adjusted Field Sites card layout to show site name, field period, and concise data summary beside a larger image.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Enhance Seosomun field site
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2706,6 +2706,70 @@
       <c r="F64" t="inlineStr">
         <is>
           <t>Added Arduino to Programming and NI DIAdem to the Data / DAQ skills category.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Enhance Seosomun Overpass field site</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Added field period, measurement configuration, system overview image, and deployment-focused text from the Seosomun reference PDF while excluding data-analysis results.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Mention Seosomun deployment in bridge monitoring project</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Updated the bridge monitoring project field deployment section to include Seosomun Overpass and its cloud-connected measurement setup.</t>
         </is>
       </c>
     </row>
@@ -3624,7 +3688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4513,6 +4577,28 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Enhanced Seosomun Overpass field site</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Used the Seosomun Overpass reference PDF to add deployment period, measurement setup, system overview image, and non-analytical system context.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Seosomun sensor placement figures
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2770,6 +2770,70 @@
       <c r="F66" t="inlineStr">
         <is>
           <t>Updated the bridge monitoring project field deployment section to include Seosomun Overpass and its cloud-connected measurement setup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Add Seosomun sensor placement figures</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Replaced the Seosomun card image with an annotated installation overview and added a second sensor-installation detail figure to the field site page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Add Seosomun accident condolence note</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Added a short condolence sentence regarding the May 26, 2026 Seosomun Overpass demolition-site collapse accident.</t>
         </is>
       </c>
     </row>
@@ -3688,7 +3752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4599,6 +4663,28 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Added Seosomun sensor placement figures</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Updated Seosomun field site images with annotated system overview and sensor installation details, adjusted card spacing, and added a brief condolence note.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Seosomun figure captions
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2834,6 +2834,38 @@
       <c r="F68" t="inlineStr">
         <is>
           <t>Added a short condolence sentence regarding the May 26, 2026 Seosomun Overpass demolition-site collapse accident.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Convert Seosomun figure captions to English</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Updated the Seosomun installation detail figure so panel captions and added labels are in English.</t>
         </is>
       </c>
     </row>
@@ -3752,7 +3784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4685,6 +4717,28 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Updated Seosomun figure captions to English</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Regenerated the Seosomun sensor installation detail figure with English panel captions and English sensor/target labels.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Seosomun collapse reflection note
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2866,6 +2866,102 @@
       <c r="F69" t="inlineStr">
         <is>
           <t>Updated the Seosomun installation detail figure so panel captions and added labels are in English.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Add Seosomun collapse reflection note</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Added a public note reflecting on the Seosomun Overpass collapse while keeping factual wording cautious and respectful.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Add location line to field site cards</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Added a location line below each field site name and increased spacing between the date/period and data summary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Distinguish figure captions from body text</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Updated figure caption styling with a soft background and accent border so captions read separately from body paragraphs.</t>
         </is>
       </c>
     </row>
@@ -3784,7 +3880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4739,6 +4835,28 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Added Seosomun reflection note and caption styling</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Created a Seosomun Overpass collapse reflection note, added field-site card locations, improved card spacing, and made figure captions visually distinct.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Use revised Seosomun figures
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2962,6 +2962,38 @@
       <c r="F72" t="inlineStr">
         <is>
           <t>Updated figure caption styling with a soft background and accent border so captions read separately from body paragraphs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Replace Seosomun figures with user-edited PDF versions</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Regenerated Seosomun installation figures directly from the updated PDF with user-edited English captions.</t>
         </is>
       </c>
     </row>
@@ -3880,7 +3912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4857,6 +4889,28 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Replaced Seosomun figures from updated PDF</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Updated Seosomun field site figures using the revised PDF with English labels/captions provided by the user.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Choha-cheon field site
</commit_message>
<xml_diff>
--- a/website_checklist.xlsx
+++ b/website_checklist.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2994,6 +2994,70 @@
       <c r="F73" t="inlineStr">
         <is>
           <t>Regenerated Seosomun installation figures directly from the updated PDF with user-edited English captions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Add Choha-cheon Bridge field site</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Added Choha-cheon Bridge as a field site with 2022.10-present monitoring period, weekly eight-channel strain measurements, and QR-code-based data acquisition context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Field Sites</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Embed Choha-cheon system demonstration video</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Added the provided YouTube system demonstration to the Choha-cheon Bridge field site page.</t>
         </is>
       </c>
     </row>
@@ -3912,7 +3976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4911,6 +4975,28 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Added Choha-cheon Bridge field site</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Added a field site page and listing entry for Choha-cheon Bridge with QR-based data acquisition and weekly eight-channel strain monitoring.</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>User + Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>